<commit_message>
Changed files from 4 surfaces to 3, removed carpet due to incomplete data
</commit_message>
<xml_diff>
--- a/ProjectFiles/Top8Aggregated_Surface(exl).xlsx
+++ b/ProjectFiles/Top8Aggregated_Surface(exl).xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM5"/>
+  <dimension ref="A1:AM4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,485 +622,364 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Carpet</t>
+          <t>Clay</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7.94</v>
+        <v>4.38</v>
       </c>
       <c r="D2" t="n">
-        <v>2.15</v>
+        <v>2.06</v>
       </c>
       <c r="E2" t="n">
-        <v>69.89</v>
+        <v>76.64</v>
       </c>
       <c r="F2" t="n">
-        <v>42.79</v>
+        <v>48.37</v>
       </c>
       <c r="G2" t="n">
-        <v>33.96</v>
+        <v>35.23</v>
       </c>
       <c r="H2" t="n">
-        <v>15.11</v>
+        <v>15.82</v>
       </c>
       <c r="I2" t="n">
-        <v>2.57</v>
+        <v>3.62</v>
       </c>
       <c r="J2" t="n">
-        <v>3.64</v>
+        <v>5.42</v>
       </c>
       <c r="K2" t="n">
-        <v>77.75</v>
+        <v>86.84999999999999</v>
       </c>
       <c r="L2" t="n">
-        <v>61.28</v>
+        <v>63.27</v>
       </c>
       <c r="M2" t="n">
-        <v>80.29000000000001</v>
+        <v>74.02</v>
       </c>
       <c r="N2" t="n">
-        <v>57.23</v>
+        <v>57.29</v>
       </c>
       <c r="O2" t="n">
-        <v>11.44</v>
+        <v>12.32</v>
       </c>
       <c r="P2" t="n">
-        <v>30.05</v>
+        <v>38.13</v>
       </c>
       <c r="Q2" t="n">
-        <v>54.82</v>
+        <v>56.35</v>
       </c>
       <c r="R2" t="n">
-        <v>6.28</v>
+        <v>3.4</v>
       </c>
       <c r="S2" t="n">
-        <v>2.76</v>
+        <v>2.71</v>
       </c>
       <c r="T2" t="n">
-        <v>72.29000000000001</v>
+        <v>80.59</v>
       </c>
       <c r="U2" t="n">
-        <v>42.18</v>
+        <v>48.86</v>
       </c>
       <c r="V2" t="n">
-        <v>29.78</v>
+        <v>30.67</v>
       </c>
       <c r="W2" t="n">
-        <v>13.82</v>
+        <v>14.12</v>
       </c>
       <c r="X2" t="n">
-        <v>3.76</v>
+        <v>5.3</v>
       </c>
       <c r="Y2" t="n">
-        <v>6.91</v>
+        <v>9.85</v>
       </c>
       <c r="Z2" t="n">
-        <v>64.42</v>
+        <v>70.37</v>
       </c>
       <c r="AA2" t="n">
-        <v>58.53</v>
+        <v>60.5</v>
       </c>
       <c r="AB2" t="n">
-        <v>69.95</v>
+        <v>61.87</v>
       </c>
       <c r="AC2" t="n">
-        <v>45.18</v>
+        <v>43.65</v>
       </c>
       <c r="AD2" t="n">
-        <v>11.27</v>
+        <v>12.14</v>
       </c>
       <c r="AE2" t="n">
-        <v>19.72</v>
+        <v>25.98</v>
       </c>
       <c r="AF2" t="n">
-        <v>42.77</v>
+        <v>42.71</v>
       </c>
       <c r="AG2" t="n">
-        <v>54.7</v>
+        <v>55.24</v>
       </c>
       <c r="AH2" t="n">
-        <v>2.75</v>
+        <v>2.77</v>
       </c>
       <c r="AI2" t="n">
-        <v>10.33</v>
+        <v>12.15</v>
       </c>
       <c r="AJ2" t="n">
-        <v>12.05</v>
+        <v>13.64</v>
       </c>
       <c r="AK2" t="n">
-        <v>55.73</v>
+        <v>55.85</v>
       </c>
       <c r="AL2" t="n">
-        <v>34.5</v>
+        <v>35.56</v>
       </c>
       <c r="AM2" t="n">
-        <v>16.35</v>
+        <v>13.36</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Clay</t>
+          <t>Grass</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4.38</v>
+        <v>13.37</v>
       </c>
       <c r="D3" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="E3" t="n">
+        <v>105.94</v>
+      </c>
+      <c r="F3" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="G3" t="n">
+        <v>54.18</v>
+      </c>
+      <c r="H3" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="J3" t="n">
+        <v>4.95</v>
+      </c>
+      <c r="K3" t="n">
+        <v>120.24</v>
+      </c>
+      <c r="L3" t="n">
+        <v>64.15000000000001</v>
+      </c>
+      <c r="M3" t="n">
+        <v>80.78</v>
+      </c>
+      <c r="N3" t="n">
+        <v>58.75</v>
+      </c>
+      <c r="O3" t="n">
+        <v>17.83</v>
+      </c>
+      <c r="P3" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>53.38</v>
+      </c>
+      <c r="R3" t="n">
+        <v>9.050000000000001</v>
+      </c>
+      <c r="S3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="T3" t="n">
+        <v>114</v>
+      </c>
+      <c r="U3" t="n">
+        <v>71.01000000000001</v>
+      </c>
+      <c r="V3" t="n">
+        <v>49.49</v>
+      </c>
+      <c r="W3" t="n">
+        <v>20.37</v>
+      </c>
+      <c r="X3" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>10.59</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>99.70999999999999</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>62.09</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>68.81</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>46.62</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>17.51</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>19.22</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>41.25</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>54.68</v>
+      </c>
+      <c r="AH3" t="n">
         <v>2.06</v>
       </c>
-      <c r="E3" t="n">
-        <v>76.64</v>
-      </c>
-      <c r="F3" t="n">
-        <v>48.37</v>
-      </c>
-      <c r="G3" t="n">
-        <v>35.23</v>
-      </c>
-      <c r="H3" t="n">
-        <v>15.82</v>
-      </c>
-      <c r="I3" t="n">
-        <v>3.62</v>
-      </c>
-      <c r="J3" t="n">
-        <v>5.42</v>
-      </c>
-      <c r="K3" t="n">
-        <v>86.84999999999999</v>
-      </c>
-      <c r="L3" t="n">
-        <v>63.27</v>
-      </c>
-      <c r="M3" t="n">
-        <v>74.02</v>
-      </c>
-      <c r="N3" t="n">
-        <v>57.29</v>
-      </c>
-      <c r="O3" t="n">
-        <v>12.32</v>
-      </c>
-      <c r="P3" t="n">
-        <v>38.13</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>56.35</v>
-      </c>
-      <c r="R3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="S3" t="n">
-        <v>2.71</v>
-      </c>
-      <c r="T3" t="n">
-        <v>80.59</v>
-      </c>
-      <c r="U3" t="n">
-        <v>48.86</v>
-      </c>
-      <c r="V3" t="n">
-        <v>30.67</v>
-      </c>
-      <c r="W3" t="n">
-        <v>14.12</v>
-      </c>
-      <c r="X3" t="n">
-        <v>5.3</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>9.85</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>70.37</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>60.5</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>61.87</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>43.65</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>12.14</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>25.98</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>42.71</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>55.24</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>2.77</v>
-      </c>
       <c r="AI3" t="n">
-        <v>12.15</v>
+        <v>11.97</v>
       </c>
       <c r="AJ3" t="n">
-        <v>13.64</v>
+        <v>12.13</v>
       </c>
       <c r="AK3" t="n">
-        <v>55.85</v>
+        <v>59.38</v>
       </c>
       <c r="AL3" t="n">
-        <v>35.56</v>
+        <v>31.75</v>
       </c>
       <c r="AM3" t="n">
-        <v>13.36</v>
+        <v>13.47</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>13.37</v>
+        <v>7.95</v>
       </c>
       <c r="D4" t="n">
-        <v>3.07</v>
+        <v>2.52</v>
       </c>
       <c r="E4" t="n">
-        <v>105.94</v>
+        <v>78.14</v>
       </c>
       <c r="F4" t="n">
-        <v>67.8</v>
+        <v>48.1</v>
       </c>
       <c r="G4" t="n">
-        <v>54.18</v>
+        <v>37.22</v>
       </c>
       <c r="H4" t="n">
-        <v>21.91</v>
+        <v>16.96</v>
       </c>
       <c r="I4" t="n">
-        <v>3.54</v>
+        <v>3.12</v>
       </c>
       <c r="J4" t="n">
-        <v>4.95</v>
+        <v>4.5</v>
       </c>
       <c r="K4" t="n">
-        <v>120.24</v>
+        <v>88.15000000000001</v>
       </c>
       <c r="L4" t="n">
-        <v>64.15000000000001</v>
+        <v>61.7</v>
       </c>
       <c r="M4" t="n">
-        <v>80.78</v>
+        <v>78.45</v>
       </c>
       <c r="N4" t="n">
-        <v>58.75</v>
+        <v>57.62</v>
       </c>
       <c r="O4" t="n">
-        <v>17.83</v>
+        <v>12.77</v>
       </c>
       <c r="P4" t="n">
-        <v>31.19</v>
+        <v>33.16</v>
       </c>
       <c r="Q4" t="n">
-        <v>53.38</v>
+        <v>54.68</v>
       </c>
       <c r="R4" t="n">
-        <v>9.050000000000001</v>
+        <v>5.87</v>
       </c>
       <c r="S4" t="n">
-        <v>4.2</v>
+        <v>3.35</v>
       </c>
       <c r="T4" t="n">
-        <v>114</v>
+        <v>82.54000000000001</v>
       </c>
       <c r="U4" t="n">
-        <v>71.01000000000001</v>
+        <v>49.02</v>
       </c>
       <c r="V4" t="n">
-        <v>49.49</v>
+        <v>33.13</v>
       </c>
       <c r="W4" t="n">
-        <v>20.37</v>
+        <v>15.44</v>
       </c>
       <c r="X4" t="n">
-        <v>6.19</v>
+        <v>4.81</v>
       </c>
       <c r="Y4" t="n">
-        <v>10.59</v>
+        <v>8.6</v>
       </c>
       <c r="Z4" t="n">
-        <v>99.70999999999999</v>
+        <v>72.53</v>
       </c>
       <c r="AA4" t="n">
-        <v>62.09</v>
+        <v>59.09</v>
       </c>
       <c r="AB4" t="n">
-        <v>68.81</v>
+        <v>66.84</v>
       </c>
       <c r="AC4" t="n">
-        <v>46.62</v>
+        <v>45.32</v>
       </c>
       <c r="AD4" t="n">
-        <v>17.51</v>
+        <v>12.53</v>
       </c>
       <c r="AE4" t="n">
-        <v>19.22</v>
+        <v>21.55</v>
       </c>
       <c r="AF4" t="n">
-        <v>41.25</v>
+        <v>42.38</v>
       </c>
       <c r="AG4" t="n">
-        <v>54.68</v>
+        <v>54.86</v>
       </c>
       <c r="AH4" t="n">
-        <v>2.06</v>
+        <v>2.61</v>
       </c>
       <c r="AI4" t="n">
-        <v>11.97</v>
+        <v>11.61</v>
       </c>
       <c r="AJ4" t="n">
-        <v>12.13</v>
+        <v>12.3</v>
       </c>
       <c r="AK4" t="n">
-        <v>59.38</v>
+        <v>57.57</v>
       </c>
       <c r="AL4" t="n">
-        <v>31.75</v>
+        <v>34.44</v>
       </c>
       <c r="AM4" t="n">
-        <v>13.47</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>7.95</v>
-      </c>
-      <c r="D5" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="E5" t="n">
-        <v>78.14</v>
-      </c>
-      <c r="F5" t="n">
-        <v>48.1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>37.22</v>
-      </c>
-      <c r="H5" t="n">
-        <v>16.96</v>
-      </c>
-      <c r="I5" t="n">
-        <v>3.12</v>
-      </c>
-      <c r="J5" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="K5" t="n">
-        <v>88.15000000000001</v>
-      </c>
-      <c r="L5" t="n">
-        <v>61.7</v>
-      </c>
-      <c r="M5" t="n">
-        <v>78.45</v>
-      </c>
-      <c r="N5" t="n">
-        <v>57.62</v>
-      </c>
-      <c r="O5" t="n">
-        <v>12.77</v>
-      </c>
-      <c r="P5" t="n">
-        <v>33.16</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>54.68</v>
-      </c>
-      <c r="R5" t="n">
-        <v>5.87</v>
-      </c>
-      <c r="S5" t="n">
-        <v>3.35</v>
-      </c>
-      <c r="T5" t="n">
-        <v>82.54000000000001</v>
-      </c>
-      <c r="U5" t="n">
-        <v>49.02</v>
-      </c>
-      <c r="V5" t="n">
-        <v>33.13</v>
-      </c>
-      <c r="W5" t="n">
-        <v>15.44</v>
-      </c>
-      <c r="X5" t="n">
-        <v>4.81</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>8.6</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>72.53</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>59.09</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>66.84</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>45.32</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>12.53</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>21.55</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>42.38</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>54.86</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>2.61</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>11.61</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>12.3</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>57.57</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>34.44</v>
-      </c>
-      <c r="AM5" t="n">
         <v>13.71</v>
       </c>
     </row>

</xml_diff>